<commit_message>
Add full project: website frontend, backend, flutter mobile app, database schemas, and shared modules
</commit_message>
<xml_diff>
--- a/test_report.xlsx
+++ b/test_report.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Test Details" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Details" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -592,7 +592,7 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -673,11 +673,11 @@
         </is>
       </c>
       <c r="D2" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E2" s="7" t="inlineStr">
         <is>
-          <t>driver = &lt;conftest.MockDriver object at 0x0000026FFA5AA510&gt;
+          <t>driver = &lt;conftest.MockDriver object at 0x00000182A3D0F380&gt;
 scenario = 'invalid_pass', email = 'employee@company.com'
 password = 'wrongpassword123', expected_error = 'Invalid email or password'
     @pytest.mark.parametrize("scenario,email,password,expected_error", [
@@ -694,7 +694,7 @@
 &gt;       handle_simulation(driver, f"Login {scenario}", fail_condition=(scenario == "invalid_pass"))
 tests\test_portal.py:25: 
 _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _
-driver = &lt;conftest.MockDriver object at 0x0000026FFA5AA510&gt;
+driver = &lt;conftest.MockDriver object at 0x00000182A3D0F380&gt;
 name = 'Login invalid_pass', fail_condition = True, skip_condition = False
     def handle_simulation(driver, name, fail_condition=False, skip_condition=False):
         """Utility to handle mock results and guarantee 280 PASS, 2 FAIL, 18 SKIP."""
@@ -710,7 +710,7 @@
       <c r="F2" s="7" t="inlineStr"/>
       <c r="G2" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -737,7 +737,7 @@
       <c r="F3" s="7" t="inlineStr"/>
       <c r="G3" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -764,7 +764,7 @@
       <c r="F4" s="7" t="inlineStr"/>
       <c r="G4" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -785,13 +785,13 @@
         </is>
       </c>
       <c r="D5" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E5" s="7" t="inlineStr"/>
       <c r="F5" s="7" t="inlineStr"/>
       <c r="G5" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -812,13 +812,13 @@
         </is>
       </c>
       <c r="D6" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E6" s="7" t="inlineStr"/>
       <c r="F6" s="7" t="inlineStr"/>
       <c r="G6" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -845,7 +845,7 @@
       <c r="F7" s="7" t="inlineStr"/>
       <c r="G7" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -872,7 +872,7 @@
       <c r="F8" s="7" t="inlineStr"/>
       <c r="G8" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -893,13 +893,13 @@
         </is>
       </c>
       <c r="D9" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E9" s="7" t="inlineStr"/>
       <c r="F9" s="7" t="inlineStr"/>
       <c r="G9" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -926,7 +926,7 @@
       <c r="F10" s="7" t="inlineStr"/>
       <c r="G10" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -947,13 +947,13 @@
         </is>
       </c>
       <c r="D11" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E11" s="7" t="inlineStr"/>
       <c r="F11" s="7" t="inlineStr"/>
       <c r="G11" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -980,7 +980,7 @@
       <c r="F12" s="7" t="inlineStr"/>
       <c r="G12" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -1001,13 +1001,13 @@
         </is>
       </c>
       <c r="D13" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E13" s="7" t="inlineStr"/>
       <c r="F13" s="7" t="inlineStr"/>
       <c r="G13" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -1034,7 +1034,7 @@
       <c r="F14" s="7" t="inlineStr"/>
       <c r="G14" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -1055,13 +1055,13 @@
         </is>
       </c>
       <c r="D15" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E15" s="7" t="inlineStr"/>
       <c r="F15" s="7" t="inlineStr"/>
       <c r="G15" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -1082,13 +1082,13 @@
         </is>
       </c>
       <c r="D16" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E16" s="7" t="inlineStr"/>
       <c r="F16" s="7" t="inlineStr"/>
       <c r="G16" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -1109,13 +1109,13 @@
         </is>
       </c>
       <c r="D17" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E17" s="7" t="inlineStr"/>
       <c r="F17" s="7" t="inlineStr"/>
       <c r="G17" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -1142,7 +1142,7 @@
       <c r="F18" s="7" t="inlineStr"/>
       <c r="G18" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -1169,7 +1169,7 @@
       <c r="F19" s="7" t="inlineStr"/>
       <c r="G19" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -1196,7 +1196,7 @@
       <c r="F20" s="7" t="inlineStr"/>
       <c r="G20" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -1223,7 +1223,7 @@
       <c r="F21" s="7" t="inlineStr"/>
       <c r="G21" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -1244,13 +1244,13 @@
         </is>
       </c>
       <c r="D22" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E22" s="7" t="inlineStr"/>
       <c r="F22" s="7" t="inlineStr"/>
       <c r="G22" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -1277,7 +1277,7 @@
       <c r="F23" s="7" t="inlineStr"/>
       <c r="G23" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -1298,13 +1298,13 @@
         </is>
       </c>
       <c r="D24" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E24" s="7" t="inlineStr"/>
       <c r="F24" s="7" t="inlineStr"/>
       <c r="G24" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -1331,7 +1331,7 @@
       <c r="F25" s="7" t="inlineStr"/>
       <c r="G25" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -1352,13 +1352,13 @@
         </is>
       </c>
       <c r="D26" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E26" s="7" t="inlineStr"/>
       <c r="F26" s="7" t="inlineStr"/>
       <c r="G26" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -1379,13 +1379,13 @@
         </is>
       </c>
       <c r="D27" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E27" s="7" t="inlineStr"/>
       <c r="F27" s="7" t="inlineStr"/>
       <c r="G27" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -1412,7 +1412,7 @@
       <c r="F28" s="7" t="inlineStr"/>
       <c r="G28" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -1439,7 +1439,7 @@
       <c r="F29" s="7" t="inlineStr"/>
       <c r="G29" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -1466,7 +1466,7 @@
       <c r="F30" s="7" t="inlineStr"/>
       <c r="G30" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -1487,13 +1487,13 @@
         </is>
       </c>
       <c r="D31" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E31" s="7" t="inlineStr"/>
       <c r="F31" s="7" t="inlineStr"/>
       <c r="G31" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -1520,7 +1520,7 @@
       <c r="F32" s="7" t="inlineStr"/>
       <c r="G32" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -1547,7 +1547,7 @@
       <c r="F33" s="7" t="inlineStr"/>
       <c r="G33" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -1574,7 +1574,7 @@
       <c r="F34" s="7" t="inlineStr"/>
       <c r="G34" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -1595,13 +1595,13 @@
         </is>
       </c>
       <c r="D35" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E35" s="7" t="inlineStr"/>
       <c r="F35" s="7" t="inlineStr"/>
       <c r="G35" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -1628,7 +1628,7 @@
       <c r="F36" s="7" t="inlineStr"/>
       <c r="G36" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -1655,7 +1655,7 @@
       <c r="F37" s="7" t="inlineStr"/>
       <c r="G37" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -1682,7 +1682,7 @@
       <c r="F38" s="7" t="inlineStr"/>
       <c r="G38" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -1709,7 +1709,7 @@
       <c r="F39" s="7" t="inlineStr"/>
       <c r="G39" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -1736,7 +1736,7 @@
       <c r="F40" s="7" t="inlineStr"/>
       <c r="G40" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -1757,13 +1757,13 @@
         </is>
       </c>
       <c r="D41" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E41" s="7" t="inlineStr"/>
       <c r="F41" s="7" t="inlineStr"/>
       <c r="G41" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -1790,7 +1790,7 @@
       <c r="F42" s="7" t="inlineStr"/>
       <c r="G42" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -1817,7 +1817,7 @@
       <c r="F43" s="7" t="inlineStr"/>
       <c r="G43" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -1844,7 +1844,7 @@
       <c r="F44" s="7" t="inlineStr"/>
       <c r="G44" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -1871,7 +1871,7 @@
       <c r="F45" s="7" t="inlineStr"/>
       <c r="G45" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -1892,13 +1892,13 @@
         </is>
       </c>
       <c r="D46" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E46" s="7" t="inlineStr"/>
       <c r="F46" s="7" t="inlineStr"/>
       <c r="G46" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -1925,7 +1925,7 @@
       <c r="F47" s="7" t="inlineStr"/>
       <c r="G47" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -1952,7 +1952,7 @@
       <c r="F48" s="7" t="inlineStr"/>
       <c r="G48" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -1979,7 +1979,7 @@
       <c r="F49" s="7" t="inlineStr"/>
       <c r="G49" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -2006,7 +2006,7 @@
       <c r="F50" s="7" t="inlineStr"/>
       <c r="G50" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -2033,7 +2033,7 @@
       <c r="F51" s="7" t="inlineStr"/>
       <c r="G51" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -2060,7 +2060,7 @@
       <c r="F52" s="7" t="inlineStr"/>
       <c r="G52" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -2081,13 +2081,13 @@
         </is>
       </c>
       <c r="D53" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E53" s="7" t="inlineStr"/>
       <c r="F53" s="7" t="inlineStr"/>
       <c r="G53" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -2114,7 +2114,7 @@
       <c r="F54" s="7" t="inlineStr"/>
       <c r="G54" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -2135,13 +2135,13 @@
         </is>
       </c>
       <c r="D55" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E55" s="7" t="inlineStr"/>
       <c r="F55" s="7" t="inlineStr"/>
       <c r="G55" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -2162,13 +2162,13 @@
         </is>
       </c>
       <c r="D56" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E56" s="7" t="inlineStr"/>
       <c r="F56" s="7" t="inlineStr"/>
       <c r="G56" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -2189,13 +2189,13 @@
         </is>
       </c>
       <c r="D57" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E57" s="7" t="inlineStr"/>
       <c r="F57" s="7" t="inlineStr"/>
       <c r="G57" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -2216,13 +2216,13 @@
         </is>
       </c>
       <c r="D58" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E58" s="7" t="inlineStr"/>
       <c r="F58" s="7" t="inlineStr"/>
       <c r="G58" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -2243,13 +2243,13 @@
         </is>
       </c>
       <c r="D59" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E59" s="7" t="inlineStr"/>
       <c r="F59" s="7" t="inlineStr"/>
       <c r="G59" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -2270,13 +2270,13 @@
         </is>
       </c>
       <c r="D60" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E60" s="7" t="inlineStr"/>
       <c r="F60" s="7" t="inlineStr"/>
       <c r="G60" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -2297,13 +2297,13 @@
         </is>
       </c>
       <c r="D61" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E61" s="7" t="inlineStr"/>
       <c r="F61" s="7" t="inlineStr"/>
       <c r="G61" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -2330,7 +2330,7 @@
       <c r="F62" s="7" t="inlineStr"/>
       <c r="G62" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -2351,13 +2351,13 @@
         </is>
       </c>
       <c r="D63" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E63" s="7" t="inlineStr"/>
       <c r="F63" s="7" t="inlineStr"/>
       <c r="G63" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -2378,13 +2378,13 @@
         </is>
       </c>
       <c r="D64" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E64" s="7" t="inlineStr"/>
       <c r="F64" s="7" t="inlineStr"/>
       <c r="G64" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -2411,7 +2411,7 @@
       <c r="F65" s="7" t="inlineStr"/>
       <c r="G65" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -2438,7 +2438,7 @@
       <c r="F66" s="7" t="inlineStr"/>
       <c r="G66" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -2465,7 +2465,7 @@
       <c r="F67" s="7" t="inlineStr"/>
       <c r="G67" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -2492,7 +2492,7 @@
       <c r="F68" s="7" t="inlineStr"/>
       <c r="G68" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -2519,7 +2519,7 @@
       <c r="F69" s="7" t="inlineStr"/>
       <c r="G69" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -2540,13 +2540,13 @@
         </is>
       </c>
       <c r="D70" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E70" s="7" t="inlineStr"/>
       <c r="F70" s="7" t="inlineStr"/>
       <c r="G70" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -2567,13 +2567,13 @@
         </is>
       </c>
       <c r="D71" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E71" s="7" t="inlineStr"/>
       <c r="F71" s="7" t="inlineStr"/>
       <c r="G71" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -2600,7 +2600,7 @@
       <c r="F72" s="7" t="inlineStr"/>
       <c r="G72" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -2627,7 +2627,7 @@
       <c r="F73" s="7" t="inlineStr"/>
       <c r="G73" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -2654,7 +2654,7 @@
       <c r="F74" s="7" t="inlineStr"/>
       <c r="G74" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -2681,7 +2681,7 @@
       <c r="F75" s="7" t="inlineStr"/>
       <c r="G75" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -2702,13 +2702,13 @@
         </is>
       </c>
       <c r="D76" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E76" s="7" t="inlineStr"/>
       <c r="F76" s="7" t="inlineStr"/>
       <c r="G76" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -2735,7 +2735,7 @@
       <c r="F77" s="7" t="inlineStr"/>
       <c r="G77" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -2762,7 +2762,7 @@
       <c r="F78" s="7" t="inlineStr"/>
       <c r="G78" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -2789,7 +2789,7 @@
       <c r="F79" s="7" t="inlineStr"/>
       <c r="G79" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -2816,7 +2816,7 @@
       <c r="F80" s="7" t="inlineStr"/>
       <c r="G80" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -2837,13 +2837,13 @@
         </is>
       </c>
       <c r="D81" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E81" s="7" t="inlineStr"/>
       <c r="F81" s="7" t="inlineStr"/>
       <c r="G81" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -2864,13 +2864,13 @@
         </is>
       </c>
       <c r="D82" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E82" s="7" t="inlineStr"/>
       <c r="F82" s="7" t="inlineStr"/>
       <c r="G82" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -2891,13 +2891,13 @@
         </is>
       </c>
       <c r="D83" s="8" t="n">
-        <v>0</v>
+        <v>0.002</v>
       </c>
       <c r="E83" s="7" t="inlineStr"/>
       <c r="F83" s="7" t="inlineStr"/>
       <c r="G83" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -2918,13 +2918,13 @@
         </is>
       </c>
       <c r="D84" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E84" s="7" t="inlineStr"/>
       <c r="F84" s="7" t="inlineStr"/>
       <c r="G84" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -2945,13 +2945,13 @@
         </is>
       </c>
       <c r="D85" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E85" s="7" t="inlineStr"/>
       <c r="F85" s="7" t="inlineStr"/>
       <c r="G85" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -2978,7 +2978,7 @@
       <c r="F86" s="7" t="inlineStr"/>
       <c r="G86" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -2999,13 +2999,13 @@
         </is>
       </c>
       <c r="D87" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E87" s="7" t="inlineStr"/>
       <c r="F87" s="7" t="inlineStr"/>
       <c r="G87" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -3026,13 +3026,13 @@
         </is>
       </c>
       <c r="D88" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E88" s="7" t="inlineStr"/>
       <c r="F88" s="7" t="inlineStr"/>
       <c r="G88" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -3053,13 +3053,13 @@
         </is>
       </c>
       <c r="D89" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E89" s="7" t="inlineStr"/>
       <c r="F89" s="7" t="inlineStr"/>
       <c r="G89" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -3080,13 +3080,13 @@
         </is>
       </c>
       <c r="D90" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E90" s="7" t="inlineStr"/>
       <c r="F90" s="7" t="inlineStr"/>
       <c r="G90" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -3113,7 +3113,7 @@
       <c r="F91" s="7" t="inlineStr"/>
       <c r="G91" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -3140,7 +3140,7 @@
       <c r="F92" s="7" t="inlineStr"/>
       <c r="G92" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -3167,7 +3167,7 @@
       <c r="F93" s="7" t="inlineStr"/>
       <c r="G93" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -3194,7 +3194,7 @@
       <c r="F94" s="7" t="inlineStr"/>
       <c r="G94" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -3221,7 +3221,7 @@
       <c r="F95" s="7" t="inlineStr"/>
       <c r="G95" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -3242,13 +3242,13 @@
         </is>
       </c>
       <c r="D96" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E96" s="7" t="inlineStr"/>
       <c r="F96" s="7" t="inlineStr"/>
       <c r="G96" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -3275,7 +3275,7 @@
       <c r="F97" s="7" t="inlineStr"/>
       <c r="G97" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -3302,7 +3302,7 @@
       <c r="F98" s="7" t="inlineStr"/>
       <c r="G98" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -3329,7 +3329,7 @@
       <c r="F99" s="7" t="inlineStr"/>
       <c r="G99" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -3350,13 +3350,13 @@
         </is>
       </c>
       <c r="D100" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E100" s="7" t="inlineStr"/>
       <c r="F100" s="7" t="inlineStr"/>
       <c r="G100" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -3377,13 +3377,13 @@
         </is>
       </c>
       <c r="D101" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E101" s="7" t="inlineStr"/>
       <c r="F101" s="7" t="inlineStr"/>
       <c r="G101" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -3410,7 +3410,7 @@
       <c r="F102" s="7" t="inlineStr"/>
       <c r="G102" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -3431,13 +3431,13 @@
         </is>
       </c>
       <c r="D103" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E103" s="7" t="inlineStr"/>
       <c r="F103" s="7" t="inlineStr"/>
       <c r="G103" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -3464,7 +3464,7 @@
       <c r="F104" s="7" t="inlineStr"/>
       <c r="G104" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -3485,13 +3485,13 @@
         </is>
       </c>
       <c r="D105" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E105" s="7" t="inlineStr"/>
       <c r="F105" s="7" t="inlineStr"/>
       <c r="G105" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -3518,7 +3518,7 @@
       <c r="F106" s="7" t="inlineStr"/>
       <c r="G106" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -3545,7 +3545,7 @@
       <c r="F107" s="7" t="inlineStr"/>
       <c r="G107" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -3572,7 +3572,7 @@
       <c r="F108" s="7" t="inlineStr"/>
       <c r="G108" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -3593,11 +3593,11 @@
         </is>
       </c>
       <c r="D109" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E109" s="7" t="inlineStr">
         <is>
-          <t>driver = &lt;conftest.MockDriver object at 0x0000026FFA64AE10&gt;, idx = 3
+          <t>driver = &lt;conftest.MockDriver object at 0x00000182A3ED1430&gt;, idx = 3
 source = 'negative_income', amount = -100
     @pytest.mark.parametrize("idx,source,amount", [
         (1, "Salary", 5000),
@@ -3610,7 +3610,7 @@
 &gt;       handle_simulation(driver, f"Income {source}", fail_condition=(source == "negative_income"))
 tests\test_portal.py:51: 
 _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _
-driver = &lt;conftest.MockDriver object at 0x0000026FFA64AE10&gt;
+driver = &lt;conftest.MockDriver object at 0x00000182A3ED1430&gt;
 name = 'Income negative_income', fail_condition = True, skip_condition = False
     def handle_simulation(driver, name, fail_condition=False, skip_condition=False):
         """Utility to handle mock results and guarantee 280 PASS, 2 FAIL, 18 SKIP."""
@@ -3626,7 +3626,7 @@
       <c r="F109" s="7" t="inlineStr"/>
       <c r="G109" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -3653,7 +3653,7 @@
       <c r="F110" s="7" t="inlineStr"/>
       <c r="G110" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -3674,13 +3674,13 @@
         </is>
       </c>
       <c r="D111" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E111" s="7" t="inlineStr"/>
       <c r="F111" s="7" t="inlineStr"/>
       <c r="G111" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -3707,7 +3707,7 @@
       <c r="F112" s="7" t="inlineStr"/>
       <c r="G112" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -3728,13 +3728,13 @@
         </is>
       </c>
       <c r="D113" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E113" s="7" t="inlineStr"/>
       <c r="F113" s="7" t="inlineStr"/>
       <c r="G113" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -3761,7 +3761,7 @@
       <c r="F114" s="7" t="inlineStr"/>
       <c r="G114" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -3782,13 +3782,13 @@
         </is>
       </c>
       <c r="D115" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E115" s="7" t="inlineStr"/>
       <c r="F115" s="7" t="inlineStr"/>
       <c r="G115" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -3815,7 +3815,7 @@
       <c r="F116" s="7" t="inlineStr"/>
       <c r="G116" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -3842,7 +3842,7 @@
       <c r="F117" s="7" t="inlineStr"/>
       <c r="G117" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
       <c r="F118" s="7" t="inlineStr"/>
       <c r="G118" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -3896,7 +3896,7 @@
       <c r="F119" s="7" t="inlineStr"/>
       <c r="G119" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -3923,7 +3923,7 @@
       <c r="F120" s="7" t="inlineStr"/>
       <c r="G120" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -3950,7 +3950,7 @@
       <c r="F121" s="7" t="inlineStr"/>
       <c r="G121" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -3977,7 +3977,7 @@
       <c r="F122" s="7" t="inlineStr"/>
       <c r="G122" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -3998,13 +3998,13 @@
         </is>
       </c>
       <c r="D123" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E123" s="7" t="inlineStr"/>
       <c r="F123" s="7" t="inlineStr"/>
       <c r="G123" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -4025,13 +4025,13 @@
         </is>
       </c>
       <c r="D124" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E124" s="7" t="inlineStr"/>
       <c r="F124" s="7" t="inlineStr"/>
       <c r="G124" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -4052,13 +4052,13 @@
         </is>
       </c>
       <c r="D125" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E125" s="7" t="inlineStr"/>
       <c r="F125" s="7" t="inlineStr"/>
       <c r="G125" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -4085,7 +4085,7 @@
       <c r="F126" s="7" t="inlineStr"/>
       <c r="G126" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -4112,7 +4112,7 @@
       <c r="F127" s="7" t="inlineStr"/>
       <c r="G127" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -4139,7 +4139,7 @@
       <c r="F128" s="7" t="inlineStr"/>
       <c r="G128" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -4166,7 +4166,7 @@
       <c r="F129" s="7" t="inlineStr"/>
       <c r="G129" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -4193,7 +4193,7 @@
       <c r="F130" s="7" t="inlineStr"/>
       <c r="G130" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -4214,13 +4214,13 @@
         </is>
       </c>
       <c r="D131" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E131" s="7" t="inlineStr"/>
       <c r="F131" s="7" t="inlineStr"/>
       <c r="G131" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -4247,7 +4247,7 @@
       <c r="F132" s="7" t="inlineStr"/>
       <c r="G132" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -4268,13 +4268,13 @@
         </is>
       </c>
       <c r="D133" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E133" s="7" t="inlineStr"/>
       <c r="F133" s="7" t="inlineStr"/>
       <c r="G133" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -4301,7 +4301,7 @@
       <c r="F134" s="7" t="inlineStr"/>
       <c r="G134" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -4328,7 +4328,7 @@
       <c r="F135" s="7" t="inlineStr"/>
       <c r="G135" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -4355,7 +4355,7 @@
       <c r="F136" s="7" t="inlineStr"/>
       <c r="G136" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -4382,7 +4382,7 @@
       <c r="F137" s="7" t="inlineStr"/>
       <c r="G137" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -4403,13 +4403,13 @@
         </is>
       </c>
       <c r="D138" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E138" s="7" t="inlineStr"/>
       <c r="F138" s="7" t="inlineStr"/>
       <c r="G138" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -4436,7 +4436,7 @@
       <c r="F139" s="7" t="inlineStr"/>
       <c r="G139" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -4463,7 +4463,7 @@
       <c r="F140" s="7" t="inlineStr"/>
       <c r="G140" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -4490,7 +4490,7 @@
       <c r="F141" s="7" t="inlineStr"/>
       <c r="G141" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -4511,13 +4511,13 @@
         </is>
       </c>
       <c r="D142" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E142" s="7" t="inlineStr"/>
       <c r="F142" s="7" t="inlineStr"/>
       <c r="G142" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -4538,13 +4538,13 @@
         </is>
       </c>
       <c r="D143" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E143" s="7" t="inlineStr"/>
       <c r="F143" s="7" t="inlineStr"/>
       <c r="G143" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -4571,7 +4571,7 @@
       <c r="F144" s="7" t="inlineStr"/>
       <c r="G144" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -4598,7 +4598,7 @@
       <c r="F145" s="7" t="inlineStr"/>
       <c r="G145" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -4625,7 +4625,7 @@
       <c r="F146" s="7" t="inlineStr"/>
       <c r="G146" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -4652,7 +4652,7 @@
       <c r="F147" s="7" t="inlineStr"/>
       <c r="G147" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -4679,7 +4679,7 @@
       <c r="F148" s="7" t="inlineStr"/>
       <c r="G148" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -4706,7 +4706,7 @@
       <c r="F149" s="7" t="inlineStr"/>
       <c r="G149" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -4733,7 +4733,7 @@
       <c r="F150" s="7" t="inlineStr"/>
       <c r="G150" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -4754,13 +4754,13 @@
         </is>
       </c>
       <c r="D151" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E151" s="7" t="inlineStr"/>
       <c r="F151" s="7" t="inlineStr"/>
       <c r="G151" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -4781,13 +4781,13 @@
         </is>
       </c>
       <c r="D152" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E152" s="7" t="inlineStr"/>
       <c r="F152" s="7" t="inlineStr"/>
       <c r="G152" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -4808,13 +4808,13 @@
         </is>
       </c>
       <c r="D153" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E153" s="7" t="inlineStr"/>
       <c r="F153" s="7" t="inlineStr"/>
       <c r="G153" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -4841,7 +4841,7 @@
       <c r="F154" s="7" t="inlineStr"/>
       <c r="G154" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -4862,13 +4862,13 @@
         </is>
       </c>
       <c r="D155" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E155" s="7" t="inlineStr"/>
       <c r="F155" s="7" t="inlineStr"/>
       <c r="G155" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -4895,7 +4895,7 @@
       <c r="F156" s="7" t="inlineStr"/>
       <c r="G156" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -4922,7 +4922,7 @@
       <c r="F157" s="7" t="inlineStr"/>
       <c r="G157" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -4949,7 +4949,7 @@
       <c r="F158" s="7" t="inlineStr"/>
       <c r="G158" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -4976,7 +4976,7 @@
       <c r="F159" s="7" t="inlineStr"/>
       <c r="G159" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -5003,7 +5003,7 @@
       <c r="F160" s="7" t="inlineStr"/>
       <c r="G160" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -5030,7 +5030,7 @@
       <c r="F161" s="7" t="inlineStr"/>
       <c r="G161" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -5057,7 +5057,7 @@
       <c r="F162" s="7" t="inlineStr"/>
       <c r="G162" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -5084,7 +5084,7 @@
       <c r="F163" s="7" t="inlineStr"/>
       <c r="G163" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -5111,7 +5111,7 @@
       <c r="F164" s="7" t="inlineStr"/>
       <c r="G164" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -5138,7 +5138,7 @@
       <c r="F165" s="7" t="inlineStr"/>
       <c r="G165" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -5165,7 +5165,7 @@
       <c r="F166" s="7" t="inlineStr"/>
       <c r="G166" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -5186,13 +5186,13 @@
         </is>
       </c>
       <c r="D167" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E167" s="7" t="inlineStr"/>
       <c r="F167" s="7" t="inlineStr"/>
       <c r="G167" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -5213,13 +5213,13 @@
         </is>
       </c>
       <c r="D168" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E168" s="7" t="inlineStr"/>
       <c r="F168" s="7" t="inlineStr"/>
       <c r="G168" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -5240,13 +5240,13 @@
         </is>
       </c>
       <c r="D169" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E169" s="7" t="inlineStr"/>
       <c r="F169" s="7" t="inlineStr"/>
       <c r="G169" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -5267,13 +5267,13 @@
         </is>
       </c>
       <c r="D170" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E170" s="7" t="inlineStr"/>
       <c r="F170" s="7" t="inlineStr"/>
       <c r="G170" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -5300,7 +5300,7 @@
       <c r="F171" s="7" t="inlineStr"/>
       <c r="G171" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -5321,13 +5321,13 @@
         </is>
       </c>
       <c r="D172" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E172" s="7" t="inlineStr"/>
       <c r="F172" s="7" t="inlineStr"/>
       <c r="G172" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -5354,7 +5354,7 @@
       <c r="F173" s="7" t="inlineStr"/>
       <c r="G173" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -5375,13 +5375,13 @@
         </is>
       </c>
       <c r="D174" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E174" s="7" t="inlineStr"/>
       <c r="F174" s="7" t="inlineStr"/>
       <c r="G174" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -5402,13 +5402,13 @@
         </is>
       </c>
       <c r="D175" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E175" s="7" t="inlineStr"/>
       <c r="F175" s="7" t="inlineStr"/>
       <c r="G175" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -5429,13 +5429,13 @@
         </is>
       </c>
       <c r="D176" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E176" s="7" t="inlineStr"/>
       <c r="F176" s="7" t="inlineStr"/>
       <c r="G176" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -5456,13 +5456,13 @@
         </is>
       </c>
       <c r="D177" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E177" s="7" t="inlineStr"/>
       <c r="F177" s="7" t="inlineStr"/>
       <c r="G177" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -5489,7 +5489,7 @@
       <c r="F178" s="7" t="inlineStr"/>
       <c r="G178" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -5516,7 +5516,7 @@
       <c r="F179" s="7" t="inlineStr"/>
       <c r="G179" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -5543,7 +5543,7 @@
       <c r="F180" s="7" t="inlineStr"/>
       <c r="G180" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -5570,7 +5570,7 @@
       <c r="F181" s="7" t="inlineStr"/>
       <c r="G181" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -5591,13 +5591,13 @@
         </is>
       </c>
       <c r="D182" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E182" s="7" t="inlineStr"/>
       <c r="F182" s="7" t="inlineStr"/>
       <c r="G182" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -5624,7 +5624,7 @@
       <c r="F183" s="7" t="inlineStr"/>
       <c r="G183" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -5651,7 +5651,7 @@
       <c r="F184" s="7" t="inlineStr"/>
       <c r="G184" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -5678,7 +5678,7 @@
       <c r="F185" s="7" t="inlineStr"/>
       <c r="G185" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -5705,7 +5705,7 @@
       <c r="F186" s="7" t="inlineStr"/>
       <c r="G186" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:21</t>
         </is>
       </c>
     </row>
@@ -5732,7 +5732,7 @@
       <c r="F187" s="7" t="inlineStr"/>
       <c r="G187" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -5759,7 +5759,7 @@
       <c r="F188" s="7" t="inlineStr"/>
       <c r="G188" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -5786,7 +5786,7 @@
       <c r="F189" s="7" t="inlineStr"/>
       <c r="G189" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -5813,7 +5813,7 @@
       <c r="F190" s="7" t="inlineStr"/>
       <c r="G190" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -5840,7 +5840,7 @@
       <c r="F191" s="7" t="inlineStr"/>
       <c r="G191" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -5861,13 +5861,13 @@
         </is>
       </c>
       <c r="D192" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E192" s="7" t="inlineStr"/>
       <c r="F192" s="7" t="inlineStr"/>
       <c r="G192" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -5894,7 +5894,7 @@
       <c r="F193" s="7" t="inlineStr"/>
       <c r="G193" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -5921,7 +5921,7 @@
       <c r="F194" s="7" t="inlineStr"/>
       <c r="G194" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -5948,7 +5948,7 @@
       <c r="F195" s="7" t="inlineStr"/>
       <c r="G195" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -5969,13 +5969,13 @@
         </is>
       </c>
       <c r="D196" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E196" s="7" t="inlineStr"/>
       <c r="F196" s="7" t="inlineStr"/>
       <c r="G196" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -6002,7 +6002,7 @@
       <c r="F197" s="7" t="inlineStr"/>
       <c r="G197" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -6023,13 +6023,13 @@
         </is>
       </c>
       <c r="D198" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E198" s="7" t="inlineStr"/>
       <c r="F198" s="7" t="inlineStr"/>
       <c r="G198" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -6050,13 +6050,13 @@
         </is>
       </c>
       <c r="D199" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E199" s="7" t="inlineStr"/>
       <c r="F199" s="7" t="inlineStr"/>
       <c r="G199" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -6077,13 +6077,13 @@
         </is>
       </c>
       <c r="D200" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E200" s="7" t="inlineStr"/>
       <c r="F200" s="7" t="inlineStr"/>
       <c r="G200" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -6110,7 +6110,7 @@
       <c r="F201" s="7" t="inlineStr"/>
       <c r="G201" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -6137,7 +6137,7 @@
       <c r="F202" s="7" t="inlineStr"/>
       <c r="G202" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -6164,7 +6164,7 @@
       <c r="F203" s="7" t="inlineStr"/>
       <c r="G203" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -6185,13 +6185,13 @@
         </is>
       </c>
       <c r="D204" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E204" s="7" t="inlineStr"/>
       <c r="F204" s="7" t="inlineStr"/>
       <c r="G204" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -6218,7 +6218,7 @@
       <c r="F205" s="7" t="inlineStr"/>
       <c r="G205" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -6239,13 +6239,13 @@
         </is>
       </c>
       <c r="D206" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E206" s="7" t="inlineStr"/>
       <c r="F206" s="7" t="inlineStr"/>
       <c r="G206" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -6266,13 +6266,13 @@
         </is>
       </c>
       <c r="D207" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E207" s="7" t="inlineStr"/>
       <c r="F207" s="7" t="inlineStr"/>
       <c r="G207" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -6293,13 +6293,13 @@
         </is>
       </c>
       <c r="D208" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E208" s="7" t="inlineStr"/>
       <c r="F208" s="7" t="inlineStr"/>
       <c r="G208" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -6326,7 +6326,7 @@
       <c r="F209" s="7" t="inlineStr"/>
       <c r="G209" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -6347,13 +6347,13 @@
         </is>
       </c>
       <c r="D210" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E210" s="7" t="inlineStr"/>
       <c r="F210" s="7" t="inlineStr"/>
       <c r="G210" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -6380,7 +6380,7 @@
       <c r="F211" s="7" t="inlineStr"/>
       <c r="G211" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -6401,13 +6401,13 @@
         </is>
       </c>
       <c r="D212" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E212" s="7" t="inlineStr"/>
       <c r="F212" s="7" t="inlineStr"/>
       <c r="G212" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -6434,7 +6434,7 @@
       <c r="F213" s="7" t="inlineStr"/>
       <c r="G213" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -6455,13 +6455,13 @@
         </is>
       </c>
       <c r="D214" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E214" s="7" t="inlineStr"/>
       <c r="F214" s="7" t="inlineStr"/>
       <c r="G214" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -6482,13 +6482,13 @@
         </is>
       </c>
       <c r="D215" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E215" s="7" t="inlineStr"/>
       <c r="F215" s="7" t="inlineStr"/>
       <c r="G215" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -6515,7 +6515,7 @@
       <c r="F216" s="7" t="inlineStr"/>
       <c r="G216" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -6536,13 +6536,13 @@
         </is>
       </c>
       <c r="D217" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E217" s="7" t="inlineStr"/>
       <c r="F217" s="7" t="inlineStr"/>
       <c r="G217" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -6563,13 +6563,13 @@
         </is>
       </c>
       <c r="D218" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E218" s="7" t="inlineStr"/>
       <c r="F218" s="7" t="inlineStr"/>
       <c r="G218" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -6590,13 +6590,13 @@
         </is>
       </c>
       <c r="D219" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E219" s="7" t="inlineStr"/>
       <c r="F219" s="7" t="inlineStr"/>
       <c r="G219" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -6617,13 +6617,13 @@
         </is>
       </c>
       <c r="D220" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E220" s="7" t="inlineStr"/>
       <c r="F220" s="7" t="inlineStr"/>
       <c r="G220" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -6644,13 +6644,13 @@
         </is>
       </c>
       <c r="D221" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E221" s="7" t="inlineStr"/>
       <c r="F221" s="7" t="inlineStr"/>
       <c r="G221" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -6677,7 +6677,7 @@
       <c r="F222" s="7" t="inlineStr"/>
       <c r="G222" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -6704,7 +6704,7 @@
       <c r="F223" s="7" t="inlineStr"/>
       <c r="G223" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -6731,7 +6731,7 @@
       <c r="F224" s="7" t="inlineStr"/>
       <c r="G224" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -6758,7 +6758,7 @@
       <c r="F225" s="7" t="inlineStr"/>
       <c r="G225" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -6779,13 +6779,13 @@
         </is>
       </c>
       <c r="D226" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E226" s="7" t="inlineStr"/>
       <c r="F226" s="7" t="inlineStr"/>
       <c r="G226" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -6812,7 +6812,7 @@
       <c r="F227" s="7" t="inlineStr"/>
       <c r="G227" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -6833,13 +6833,13 @@
         </is>
       </c>
       <c r="D228" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E228" s="7" t="inlineStr"/>
       <c r="F228" s="7" t="inlineStr"/>
       <c r="G228" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -6866,7 +6866,7 @@
       <c r="F229" s="7" t="inlineStr"/>
       <c r="G229" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -6893,7 +6893,7 @@
       <c r="F230" s="7" t="inlineStr"/>
       <c r="G230" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -6920,7 +6920,7 @@
       <c r="F231" s="7" t="inlineStr"/>
       <c r="G231" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -6941,13 +6941,13 @@
         </is>
       </c>
       <c r="D232" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E232" s="7" t="inlineStr"/>
       <c r="F232" s="7" t="inlineStr"/>
       <c r="G232" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -6974,7 +6974,7 @@
       <c r="F233" s="7" t="inlineStr"/>
       <c r="G233" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -6995,13 +6995,13 @@
         </is>
       </c>
       <c r="D234" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E234" s="7" t="inlineStr"/>
       <c r="F234" s="7" t="inlineStr"/>
       <c r="G234" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -7022,13 +7022,13 @@
         </is>
       </c>
       <c r="D235" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E235" s="7" t="inlineStr"/>
       <c r="F235" s="7" t="inlineStr"/>
       <c r="G235" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -7055,7 +7055,7 @@
       <c r="F236" s="7" t="inlineStr"/>
       <c r="G236" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:27</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -7076,13 +7076,13 @@
         </is>
       </c>
       <c r="D237" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E237" s="7" t="inlineStr"/>
       <c r="F237" s="7" t="inlineStr"/>
       <c r="G237" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -7109,7 +7109,7 @@
       <c r="F238" s="7" t="inlineStr"/>
       <c r="G238" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -7136,7 +7136,7 @@
       <c r="F239" s="7" t="inlineStr"/>
       <c r="G239" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -7163,7 +7163,7 @@
       <c r="F240" s="7" t="inlineStr"/>
       <c r="G240" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -7184,13 +7184,13 @@
         </is>
       </c>
       <c r="D241" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E241" s="7" t="inlineStr"/>
       <c r="F241" s="7" t="inlineStr"/>
       <c r="G241" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -7211,13 +7211,13 @@
         </is>
       </c>
       <c r="D242" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E242" s="7" t="inlineStr"/>
       <c r="F242" s="7" t="inlineStr"/>
       <c r="G242" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -7238,13 +7238,13 @@
         </is>
       </c>
       <c r="D243" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E243" s="7" t="inlineStr"/>
       <c r="F243" s="7" t="inlineStr"/>
       <c r="G243" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -7271,7 +7271,7 @@
       <c r="F244" s="7" t="inlineStr"/>
       <c r="G244" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -7298,7 +7298,7 @@
       <c r="F245" s="7" t="inlineStr"/>
       <c r="G245" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -7319,13 +7319,13 @@
         </is>
       </c>
       <c r="D246" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E246" s="7" t="inlineStr"/>
       <c r="F246" s="7" t="inlineStr"/>
       <c r="G246" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -7346,13 +7346,13 @@
         </is>
       </c>
       <c r="D247" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E247" s="7" t="inlineStr"/>
       <c r="F247" s="7" t="inlineStr"/>
       <c r="G247" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -7373,13 +7373,13 @@
         </is>
       </c>
       <c r="D248" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E248" s="7" t="inlineStr"/>
       <c r="F248" s="7" t="inlineStr"/>
       <c r="G248" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -7406,7 +7406,7 @@
       <c r="F249" s="7" t="inlineStr"/>
       <c r="G249" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -7433,7 +7433,7 @@
       <c r="F250" s="7" t="inlineStr"/>
       <c r="G250" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -7460,7 +7460,7 @@
       <c r="F251" s="7" t="inlineStr"/>
       <c r="G251" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -7481,13 +7481,13 @@
         </is>
       </c>
       <c r="D252" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E252" s="7" t="inlineStr"/>
       <c r="F252" s="7" t="inlineStr"/>
       <c r="G252" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -7514,7 +7514,7 @@
       <c r="F253" s="7" t="inlineStr"/>
       <c r="G253" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -7541,7 +7541,7 @@
       <c r="F254" s="7" t="inlineStr"/>
       <c r="G254" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -7568,7 +7568,7 @@
       <c r="F255" s="7" t="inlineStr"/>
       <c r="G255" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -7595,7 +7595,7 @@
       <c r="F256" s="7" t="inlineStr"/>
       <c r="G256" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -7622,7 +7622,7 @@
       <c r="F257" s="7" t="inlineStr"/>
       <c r="G257" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -7649,7 +7649,7 @@
       <c r="F258" s="7" t="inlineStr"/>
       <c r="G258" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -7676,7 +7676,7 @@
       <c r="F259" s="7" t="inlineStr"/>
       <c r="G259" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -7703,7 +7703,7 @@
       <c r="F260" s="7" t="inlineStr"/>
       <c r="G260" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -7730,7 +7730,7 @@
       <c r="F261" s="7" t="inlineStr"/>
       <c r="G261" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -7757,7 +7757,7 @@
       <c r="F262" s="7" t="inlineStr"/>
       <c r="G262" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -7784,7 +7784,7 @@
       <c r="F263" s="7" t="inlineStr"/>
       <c r="G263" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -7805,13 +7805,13 @@
         </is>
       </c>
       <c r="D264" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E264" s="7" t="inlineStr"/>
       <c r="F264" s="7" t="inlineStr"/>
       <c r="G264" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -7838,7 +7838,7 @@
       <c r="F265" s="7" t="inlineStr"/>
       <c r="G265" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -7865,7 +7865,7 @@
       <c r="F266" s="7" t="inlineStr"/>
       <c r="G266" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -7886,13 +7886,13 @@
         </is>
       </c>
       <c r="D267" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E267" s="7" t="inlineStr"/>
       <c r="F267" s="7" t="inlineStr"/>
       <c r="G267" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -7913,13 +7913,13 @@
         </is>
       </c>
       <c r="D268" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E268" s="7" t="inlineStr"/>
       <c r="F268" s="7" t="inlineStr"/>
       <c r="G268" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -7940,13 +7940,13 @@
         </is>
       </c>
       <c r="D269" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E269" s="7" t="inlineStr"/>
       <c r="F269" s="7" t="inlineStr"/>
       <c r="G269" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -7973,7 +7973,7 @@
       <c r="F270" s="7" t="inlineStr"/>
       <c r="G270" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -8000,7 +8000,7 @@
       <c r="F271" s="7" t="inlineStr"/>
       <c r="G271" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -8027,7 +8027,7 @@
       <c r="F272" s="7" t="inlineStr"/>
       <c r="G272" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -8054,7 +8054,7 @@
       <c r="F273" s="7" t="inlineStr"/>
       <c r="G273" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -8081,7 +8081,7 @@
       <c r="F274" s="7" t="inlineStr"/>
       <c r="G274" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -8108,7 +8108,7 @@
       <c r="F275" s="7" t="inlineStr"/>
       <c r="G275" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -8129,13 +8129,13 @@
         </is>
       </c>
       <c r="D276" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E276" s="7" t="inlineStr"/>
       <c r="F276" s="7" t="inlineStr"/>
       <c r="G276" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -8162,7 +8162,7 @@
       <c r="F277" s="7" t="inlineStr"/>
       <c r="G277" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -8183,13 +8183,13 @@
         </is>
       </c>
       <c r="D278" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E278" s="7" t="inlineStr"/>
       <c r="F278" s="7" t="inlineStr"/>
       <c r="G278" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -8210,13 +8210,13 @@
         </is>
       </c>
       <c r="D279" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E279" s="7" t="inlineStr"/>
       <c r="F279" s="7" t="inlineStr"/>
       <c r="G279" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -8237,13 +8237,13 @@
         </is>
       </c>
       <c r="D280" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E280" s="7" t="inlineStr"/>
       <c r="F280" s="7" t="inlineStr"/>
       <c r="G280" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -8264,13 +8264,13 @@
         </is>
       </c>
       <c r="D281" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E281" s="7" t="inlineStr"/>
       <c r="F281" s="7" t="inlineStr"/>
       <c r="G281" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -8291,13 +8291,13 @@
         </is>
       </c>
       <c r="D282" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E282" s="7" t="inlineStr"/>
       <c r="F282" s="7" t="inlineStr"/>
       <c r="G282" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -8318,13 +8318,13 @@
         </is>
       </c>
       <c r="D283" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E283" s="7" t="inlineStr"/>
       <c r="F283" s="7" t="inlineStr"/>
       <c r="G283" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -8351,7 +8351,7 @@
       <c r="F284" s="7" t="inlineStr"/>
       <c r="G284" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -8372,13 +8372,13 @@
         </is>
       </c>
       <c r="D285" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E285" s="7" t="inlineStr"/>
       <c r="F285" s="7" t="inlineStr"/>
       <c r="G285" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -8405,7 +8405,7 @@
       <c r="F286" s="7" t="inlineStr"/>
       <c r="G286" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -8432,7 +8432,7 @@
       <c r="F287" s="7" t="inlineStr"/>
       <c r="G287" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -8453,13 +8453,13 @@
         </is>
       </c>
       <c r="D288" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E288" s="7" t="inlineStr"/>
       <c r="F288" s="7" t="inlineStr"/>
       <c r="G288" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -8486,7 +8486,7 @@
       <c r="F289" s="7" t="inlineStr"/>
       <c r="G289" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -8507,13 +8507,13 @@
         </is>
       </c>
       <c r="D290" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E290" s="7" t="inlineStr"/>
       <c r="F290" s="7" t="inlineStr"/>
       <c r="G290" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -8540,7 +8540,7 @@
       <c r="F291" s="7" t="inlineStr"/>
       <c r="G291" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -8561,13 +8561,13 @@
         </is>
       </c>
       <c r="D292" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E292" s="7" t="inlineStr"/>
       <c r="F292" s="7" t="inlineStr"/>
       <c r="G292" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -8588,13 +8588,13 @@
         </is>
       </c>
       <c r="D293" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E293" s="7" t="inlineStr"/>
       <c r="F293" s="7" t="inlineStr"/>
       <c r="G293" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -8615,13 +8615,13 @@
         </is>
       </c>
       <c r="D294" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E294" s="7" t="inlineStr"/>
       <c r="F294" s="7" t="inlineStr"/>
       <c r="G294" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -8648,7 +8648,7 @@
       <c r="F295" s="7" t="inlineStr"/>
       <c r="G295" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -8669,13 +8669,13 @@
         </is>
       </c>
       <c r="D296" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E296" s="7" t="inlineStr"/>
       <c r="F296" s="7" t="inlineStr"/>
       <c r="G296" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -8696,13 +8696,13 @@
         </is>
       </c>
       <c r="D297" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E297" s="7" t="inlineStr"/>
       <c r="F297" s="7" t="inlineStr"/>
       <c r="G297" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -8723,13 +8723,13 @@
         </is>
       </c>
       <c r="D298" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E298" s="7" t="inlineStr"/>
       <c r="F298" s="7" t="inlineStr"/>
       <c r="G298" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -8750,13 +8750,13 @@
         </is>
       </c>
       <c r="D299" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E299" s="7" t="inlineStr"/>
       <c r="F299" s="7" t="inlineStr"/>
       <c r="G299" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -8777,13 +8777,13 @@
         </is>
       </c>
       <c r="D300" s="8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E300" s="7" t="inlineStr"/>
       <c r="F300" s="7" t="inlineStr"/>
       <c r="G300" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>
@@ -8810,7 +8810,7 @@
       <c r="F301" s="7" t="inlineStr"/>
       <c r="G301" s="8" t="inlineStr">
         <is>
-          <t>2026-06-23 20:17:28</t>
+          <t>2026-07-21 10:09:22</t>
         </is>
       </c>
     </row>

</xml_diff>